<commit_message>
Added models for n hospitals in hr and per cap budget per region
</commit_message>
<xml_diff>
--- a/data/2026_hr_budget.xlsx
+++ b/data/2026_hr_budget.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fluffypony/Library/Mobile Documents/com~apple~CloudDocs/Documents/Galway/PROJECT/CODE/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{00E0F7E0-CB3C-E947-AF76-2F48B19F63F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C125D70-20A3-9D4F-BAD5-4DB9E732929F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="1020" windowWidth="25040" windowHeight="14880" xr2:uid="{67D40A30-2A8C-2D4F-BA08-F66AC3DD4B7A}"/>
+    <workbookView xWindow="0" yWindow="520" windowWidth="25600" windowHeight="16040" xr2:uid="{67D40A30-2A8C-2D4F-BA08-F66AC3DD4B7A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -466,22 +466,22 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
-        <v>3670</v>
+        <v>3670000</v>
       </c>
       <c r="B2" s="1">
-        <v>3395</v>
+        <v>3395000</v>
       </c>
       <c r="C2" s="1">
-        <v>2659</v>
+        <v>2659000</v>
       </c>
       <c r="D2" s="1">
-        <v>1182</v>
+        <v>1182000</v>
       </c>
       <c r="E2" s="1">
-        <v>2002</v>
+        <v>2002000</v>
       </c>
       <c r="F2" s="1">
-        <v>2512</v>
+        <v>2512000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>